<commit_message>
Add new feat Leave Type
</commit_message>
<xml_diff>
--- a/DataDesign_v1.2.xlsx
+++ b/DataDesign_v1.2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/06406dd7d2ddb8b6/Documents/NetBeansProjects/batch5_HR_Management_System/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="621" documentId="8_{B5BE63CA-D429-4CC9-972F-46B140711E92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90B7AC04-E616-42E0-88F9-815CF55BB015}"/>
+  <xr:revisionPtr revIDLastSave="622" documentId="8_{B5BE63CA-D429-4CC9-972F-46B140711E92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F835FCE-0644-4655-99AD-104DD8CF67F2}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="20" windowWidth="19180" windowHeight="11260" firstSheet="2" activeTab="4" xr2:uid="{67315DDE-2511-46DC-9E0F-5194690A2ED0}"/>
+    <workbookView xWindow="20" yWindow="20" windowWidth="19180" windowHeight="11260" firstSheet="2" activeTab="3" xr2:uid="{67315DDE-2511-46DC-9E0F-5194690A2ED0}"/>
   </bookViews>
   <sheets>
     <sheet name="Department &amp; Office" sheetId="1" r:id="rId1"/>
@@ -5500,7 +5500,7 @@
     <col min="8" max="8" width="32.36328125" customWidth="1"/>
     <col min="9" max="9" width="26.90625" customWidth="1"/>
     <col min="10" max="10" width="31.90625" customWidth="1"/>
-    <col min="11" max="11" width="24.81640625" customWidth="1"/>
+    <col min="11" max="11" width="28" customWidth="1"/>
     <col min="12" max="12" width="15.26953125" customWidth="1"/>
     <col min="13" max="13" width="22.54296875" customWidth="1"/>
     <col min="14" max="14" width="21.453125" customWidth="1"/>

</xml_diff>